<commit_message>
feat: equity issuance row tooltip explains computed origin
The Equity Issuance line on the CFS is back-computed from Δ APIC + Δ
Common Stock vs the prior historical period; for projection years it
uses the equityIssuance assumption. Because there is no direct
"Equity Issuance" UI input on the historical side, users were
confused when a non-zero value appeared (e.g. APIC 210k → 220k
shows as +10k issuance).

- Excel: cell note on the row label
- Engine UI: title tooltip + ⓘ marker on the CashFlowPage row

audit:sync: 1635/1635 ✓
export:audit:telecom: BS balanced, all 3 scenarios.

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/out-base.xlsx
+++ b/out-base.xlsx
@@ -28,6 +28,23 @@
 </workbook>
 </file>
 
+<file path=xl/comments7.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>Author</author>
+  </authors>
+  <commentList>
+    <comment ref="A37" authorId="0">
+      <text>
+        <r>
+          <t>Computed from Δ APIC + Δ Common Stock vs prior period (historical years) or equityIssuance assumption (projection years).</t>
+        </r>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1298" uniqueCount="499">
   <si>
@@ -286,7 +303,7 @@
     <t>Last Updated</t>
   </si>
   <si>
-    <t>April 27, 2026</t>
+    <t>April 28, 2026</t>
   </si>
   <si>
     <t>SECTION 3 — EGYPT REGULATORY / TAX</t>
@@ -28938,6 +28955,7 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <legacyDrawing r:id="rId2"/>
 </worksheet>
 </file>
 

</xml_diff>